<commit_message>
Made the DOB required field
</commit_message>
<xml_diff>
--- a/forms/contact/person-edit.xlsx
+++ b/forms/contact/person-edit.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="116">
   <si>
     <t>type</t>
   </si>
@@ -628,7 +628,7 @@
     <col customWidth="1" min="3" max="3" width="27.86"/>
     <col customWidth="1" min="4" max="4" width="28.71"/>
     <col customWidth="1" min="5" max="5" width="15.57"/>
-    <col customWidth="1" min="6" max="6" width="14.57"/>
+    <col customWidth="1" min="6" max="6" width="19.86"/>
     <col customWidth="1" min="7" max="7" width="19.57"/>
     <col customWidth="1" min="8" max="8" width="10.71"/>
     <col customWidth="1" min="9" max="9" width="24.14"/>
@@ -1368,7 +1368,9 @@
       <c r="D19" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="E19" s="1"/>
+      <c r="E19" s="5" t="s">
+        <v>45</v>
+      </c>
       <c r="F19" s="1"/>
       <c r="G19" s="1"/>
       <c r="H19" s="1"/>
@@ -11032,7 +11034,7 @@
       </c>
       <c r="C2" s="34" t="str">
         <f>TEXT(NOW(), "yyyy-mm-dd_HH-MM")</f>
-        <v>2020-10-06_09-33</v>
+        <v>2020-11-03_06-50</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>114</v>

</xml_diff>